<commit_message>
Add dashboard images and fix names
</commit_message>
<xml_diff>
--- a/data/Spotify_Tracks_2023_Clean.xlsx
+++ b/data/Spotify_Tracks_2023_Clean.xlsx
@@ -133,7 +133,7 @@
     <t>As It Was</t>
   </si>
   <si>
-    <t>Seï¿½ï¿½o</t>
+    <t>Se?o</t>
   </si>
   <si>
     <t>Say You Won't Let Go</t>
@@ -337,7 +337,7 @@
     <t>Adore You</t>
   </si>
   <si>
-    <t>LA CANCIï¿½</t>
+    <t>LA CANCI?</t>
   </si>
   <si>
     <t>The Real Slim Shady</t>
@@ -400,7 +400,7 @@
     <t>Why'd You Only Call Me When You're High?</t>
   </si>
   <si>
-    <t>Titi Me Preguntï¿</t>
+    <t>Titi Me Pregunt?</t>
   </si>
   <si>
     <t>Yonaguni</t>
@@ -697,7 +697,7 @@
     <t>favorite crime</t>
   </si>
   <si>
-    <t>DESPECHï¿</t>
+    <t>DESPECH?</t>
   </si>
   <si>
     <t>Bored</t>
@@ -745,7 +745,7 @@
     <t>Shakira: Bzrp Music Sessions, Vol. 53</t>
   </si>
   <si>
-    <t>Quï¿½ï¿½ Mï¿½ï¿</t>
+    <t>Qu? M?</t>
   </si>
   <si>
     <t>Left and Right (Feat. Jung Kook of BTS)</t>
@@ -778,13 +778,13 @@
     <t>A Tu Merced</t>
   </si>
   <si>
-    <t>Donï¿½ï¿½ï¿½t Bl</t>
+    <t>Don't Bl</t>
   </si>
   <si>
     <t>Reminder</t>
   </si>
   <si>
-    <t>Una Noche en Medellï¿½</t>
+    <t>Una Noche en Medell?</t>
   </si>
   <si>
     <t>Romantic Homicide</t>
@@ -802,7 +802,7 @@
     <t>Hey Mor</t>
   </si>
   <si>
-    <t>Volvï¿</t>
+    <t>Volv?</t>
   </si>
   <si>
     <t>You Right</t>
@@ -883,7 +883,7 @@
     <t>Te Felicito</t>
   </si>
   <si>
-    <t>Feliz Cumpleaï¿½ï¿½os Fe</t>
+    <t>Feliz Cumplea?os Fe</t>
   </si>
   <si>
     <t>Until I Found You (with Em Beihold) - Em Beihold Version</t>
@@ -892,7 +892,7 @@
     <t>Softcore</t>
   </si>
   <si>
-    <t>Miï¿½ï¿½n</t>
+    <t>Mi?n</t>
   </si>
   <si>
     <t>CUFF IT</t>
@@ -1072,7 +1072,7 @@
     <t>Oh My God</t>
   </si>
   <si>
-    <t>Cï¿½ï¿½</t>
+    <t>C?</t>
   </si>
   <si>
     <t>AMG</t>
@@ -1081,7 +1081,7 @@
     <t>Ferrari</t>
   </si>
   <si>
-    <t>Despuï¿½ï¿½s de la P</t>
+    <t>Despu?s de la P</t>
   </si>
   <si>
     <t>NEW MAGIC WAND</t>
@@ -1111,7 +1111,7 @@
     <t>Me and Your Mama</t>
   </si>
   <si>
-    <t>Nostï¿½ï¿½l</t>
+    <t>Nost?l</t>
   </si>
   <si>
     <t>PRC</t>
@@ -1237,7 +1237,7 @@
     <t>Punto G</t>
   </si>
   <si>
-    <t>Monotonï¿½</t>
+    <t>Monoton?</t>
   </si>
   <si>
     <t>Selfish</t>
@@ -1312,10 +1312,10 @@
     <t>Merry Christmas Everyone</t>
   </si>
   <si>
-    <t>You Belong With Me (Taylorï¿½ï¿½ï¿½s Ve</t>
-  </si>
-  <si>
-    <t>X ï¿½ï¿½LTIMA</t>
+    <t>You Belong With Me (Taylor's Ve</t>
+  </si>
+  <si>
+    <t>X ?LTIMA</t>
   </si>
   <si>
     <t>Fingers Crossed</t>
@@ -1366,13 +1366,13 @@
     <t>Music For a Sushi Restaurant</t>
   </si>
   <si>
-    <t>La Llevo Al Cielo (Ft. ï¿½ï¿½engo F</t>
+    <t>La Llevo Al Cielo (Ft. ?engo F</t>
   </si>
   <si>
     <t>STAR WALKIN' (League of Legends Worlds Anthem)</t>
   </si>
   <si>
-    <t>cï¿½ï¿½mo dormi</t>
+    <t>c?mo dormi</t>
   </si>
   <si>
     <t>Run BTS</t>
@@ -1402,7 +1402,7 @@
     <t>Dreamers [Music from the FIFA World Cup Qatar 2022 Official Soundtrack]</t>
   </si>
   <si>
-    <t>GATï¿½ï¿½</t>
+    <t>GAT?</t>
   </si>
   <si>
     <t>Ya No Somos Ni Seremos</t>
@@ -1546,7 +1546,7 @@
     <t>Forever</t>
   </si>
   <si>
-    <t xml:space="preserve">Ensï¿½ï¿½ï¿½ï¿½ame </t>
+    <t xml:space="preserve">Ens'?ame </t>
   </si>
   <si>
     <t>ULTRA SOLO REMIX</t>
@@ -1576,7 +1576,7 @@
     <t>Cooped Up (with Roddy Ricch)</t>
   </si>
   <si>
-    <t>Leï¿½</t>
+    <t>Le?</t>
   </si>
   <si>
     <t>Surface Pressure</t>
@@ -1594,10 +1594,10 @@
     <t>Attention</t>
   </si>
   <si>
-    <t xml:space="preserve">Vai Lï¿½ï¿½ Em Casa </t>
-  </si>
-  <si>
-    <t>Monï¿½ï¿½y so</t>
+    <t xml:space="preserve">Vai L? Em Casa </t>
+  </si>
+  <si>
+    <t>Mon?y so</t>
   </si>
   <si>
     <t>Bombonzinho - Ao Vivo</t>
@@ -1618,7 +1618,7 @@
     <t>Numb Little Bug</t>
   </si>
   <si>
-    <t>Esqueï¿½ï¿½a-Me Se For C</t>
+    <t>Esque?a-Me Se For C</t>
   </si>
   <si>
     <t>Moonlight</t>
@@ -1660,7 +1660,7 @@
     <t>Agosto</t>
   </si>
   <si>
-    <t>Cayï¿½ï¿½ La Noche (feat. Cruz Cafunï¿½ï¿½, Abhir Hathi, Bejo, EL IMA)</t>
+    <t>Cay? La Noche (feat. Cruz Cafun?, Abhir Hathi, Bejo, EL IMA)</t>
   </si>
   <si>
     <t>Run Rudolph Run - Single Version</t>
@@ -1696,7 +1696,7 @@
     <t>Ginseng Strip 2002</t>
   </si>
   <si>
-    <t>Malvadï¿½ï¿</t>
+    <t>Malvad?</t>
   </si>
   <si>
     <t>Plan A</t>
@@ -1720,7 +1720,7 @@
     <t>Tom's Diner</t>
   </si>
   <si>
-    <t>Quï¿½ï¿½ Ago</t>
+    <t>Qu? Ago</t>
   </si>
   <si>
     <t>Keep Driving</t>
@@ -1753,10 +1753,10 @@
     <t>Starlight</t>
   </si>
   <si>
-    <t>Evergreen (You Didnï¿½ï¿½ï¿½t Deserve Me A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">When Iï¿½ï¿½ï¿½m Gone (with Katy </t>
+    <t>Evergreen (You Didn't Deserve Me A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When I'm Gone (with Katy </t>
   </si>
   <si>
     <t>I AM WOMAN</t>
@@ -1786,7 +1786,7 @@
     <t>Betty (Get Money)</t>
   </si>
   <si>
-    <t>PLAYA DEL INGLï¿½</t>
+    <t>PLAYA DEL INGL?</t>
   </si>
   <si>
     <t>Bad Decisions (with BTS &amp; Snoop Dogg)</t>
@@ -1804,7 +1804,7 @@
     <t>WORTH NOTHING</t>
   </si>
   <si>
-    <t>El Apagï¿½</t>
+    <t>El Apag?</t>
   </si>
   <si>
     <t>MANIAC</t>
@@ -1822,13 +1822,13 @@
     <t>KICK BACK</t>
   </si>
   <si>
-    <t>Problemï¿½</t>
-  </si>
-  <si>
-    <t>Sin Seï¿½ï</t>
-  </si>
-  <si>
-    <t>DANï¿½ï¿½A</t>
+    <t>Problem?</t>
+  </si>
+  <si>
+    <t>Sin Se?</t>
+  </si>
+  <si>
+    <t>DAN?A</t>
   </si>
   <si>
     <t>Watch This - ARIZONATEARS Pluggnb Remix</t>
@@ -1927,7 +1927,7 @@
     <t>Cinema</t>
   </si>
   <si>
-    <t>Frï¿½ï¿½gil (feat. Grupo Front</t>
+    <t>Fr?gil (feat. Grupo Front</t>
   </si>
   <si>
     <t>Vampiro</t>
@@ -1969,7 +1969,7 @@
     <t>Good Looking</t>
   </si>
   <si>
-    <t>TUS Lï¿½ï¿½GR</t>
+    <t>TUS L?GR</t>
   </si>
   <si>
     <t>Escapism. - Sped Up</t>
@@ -1999,7 +1999,7 @@
     <t>Tak Segampang Itu</t>
   </si>
   <si>
-    <t>Si Te La Encuentras Por Ahï¿</t>
+    <t>Si Te La Encuentras Por Ah?</t>
   </si>
   <si>
     <t>Jingle Bells - Remastered 1999</t>
@@ -2014,7 +2014,7 @@
     <t>Would've, Could've, Should've</t>
   </si>
   <si>
-    <t>Sï¿½ï¿½</t>
+    <t>S?</t>
   </si>
   <si>
     <t>TQM</t>
@@ -2101,10 +2101,10 @@
     <t>BABY OTAKU</t>
   </si>
   <si>
-    <t>Igualito a Mi Apï¿</t>
-  </si>
-  <si>
-    <t>RUMBATï¿½</t>
+    <t>Igualito a Mi Ap?</t>
+  </si>
+  <si>
+    <t>RUMBAT?</t>
   </si>
   <si>
     <t>Antes de Perderte</t>
@@ -2278,7 +2278,7 @@
     <t>LALA</t>
   </si>
   <si>
-    <t>This Love (Taylorï¿½ï¿½ï¿½s Ve</t>
+    <t>This Love (Taylor's Ve</t>
   </si>
   <si>
     <t>die first</t>
@@ -2311,7 +2311,7 @@
     <t>Count Me Out</t>
   </si>
   <si>
-    <t>Thinkinï¿½ï¿½ï¿½ B</t>
+    <t>Thinkin' B</t>
   </si>
   <si>
     <t>LLYLM</t>
@@ -2329,7 +2329,7 @@
     <t>I AM</t>
   </si>
   <si>
-    <t>Acrï¿½ï¿½s</t>
+    <t>Acr?s</t>
   </si>
   <si>
     <t>Los del Espacio</t>
@@ -2350,7 +2350,7 @@
     <t>I Tried to Tell Y'all</t>
   </si>
   <si>
-    <t>Muï¿½ï¿½</t>
+    <t>Mu?</t>
   </si>
   <si>
     <t>Nobody Like U - From "Turning Red"</t>
@@ -2365,7 +2365,7 @@
     <t>Take Two</t>
   </si>
   <si>
-    <t>Me Arrepentï¿</t>
+    <t>Me Arrepent?</t>
   </si>
   <si>
     <t>Never Felt So Alone</t>
@@ -2383,7 +2383,7 @@
     <t>Dijeron Que No La Iba Lograr</t>
   </si>
   <si>
-    <t>Tubarï¿½ï¿½o Te</t>
+    <t>Tubar?o Te</t>
   </si>
   <si>
     <t>Popular (with Playboi Carti &amp; Madonna) - The Idol Vol. 1 (Music from the HBO Original Series)</t>
@@ -2392,7 +2392,7 @@
     <t>Poland</t>
   </si>
   <si>
-    <t>Niï¿½ï¿½a Bo</t>
+    <t>Ni?a Bo</t>
   </si>
   <si>
     <t>For Youth</t>
@@ -2404,7 +2404,7 @@
     <t>Privileged Rappers</t>
   </si>
   <si>
-    <t>Tï¿½ï¿</t>
+    <t>T?</t>
   </si>
   <si>
     <t>Love Language</t>
@@ -2422,7 +2422,7 @@
     <t>Thinking with My Dick</t>
   </si>
   <si>
-    <t>Lï¿½ï¿½ï¿</t>
+    <t>L?</t>
   </si>
   <si>
     <t>El Cielo</t>
@@ -2452,7 +2452,7 @@
     <t>I'm Not Here To Make Friends</t>
   </si>
   <si>
-    <t>Cupid ï¿½ï¿½ï¿½ Twin Ver. (FIFTY FIFTY) ï¿½ï¿½ï¿½ Spe</t>
+    <t>Cupid ' Twin Ver. (FIFTY FIFTY) ' Spe</t>
   </si>
   <si>
     <t>Right On</t>
@@ -2461,7 +2461,7 @@
     <t>Best Friends</t>
   </si>
   <si>
-    <t>Arcï¿½ï¿½ngel: Bzrp Music Sessions, Vol</t>
+    <t>Arc?ngel: Bzrp Music Sessions, Vol</t>
   </si>
   <si>
     <t>Seek &amp; Destroy</t>
@@ -2503,10 +2503,10 @@
     <t>Used (feat. Don Toliver)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sem Alianï¿½ï¿½a no </t>
-  </si>
-  <si>
-    <t>PERO Tï¿</t>
+    <t xml:space="preserve">Sem Alian?a no </t>
+  </si>
+  <si>
+    <t>PERO T?</t>
   </si>
   <si>
     <t>BackOutsideBoyz</t>
@@ -2530,7 +2530,7 @@
     <t>VAGABUNDO</t>
   </si>
   <si>
-    <t>Agudo Mï¿½ï¿½gi</t>
+    <t>Agudo M?gi</t>
   </si>
   <si>
     <t>Rosa Pastel</t>
@@ -2542,10 +2542,10 @@
     <t>Chance</t>
   </si>
   <si>
-    <t>Ainï¿½ï¿½ï¿½t Tha</t>
-  </si>
-  <si>
-    <t>Here We Goï¿½ï¿½ï¿½ Again (feat. Tyler, the Cr</t>
+    <t>Ain't Tha</t>
+  </si>
+  <si>
+    <t>Here We Go' Again (feat. Tyler, the Cr</t>
   </si>
   <si>
     <t>Special</t>
@@ -2578,7 +2578,7 @@
     <t>Do We Have A Problem?</t>
   </si>
   <si>
-    <t>Novo Balanï¿½</t>
+    <t>Novo Balan?</t>
   </si>
   <si>
     <t>DOGTOOTH</t>
@@ -2605,7 +2605,7 @@
     <t>Primera Cita</t>
   </si>
   <si>
-    <t xml:space="preserve">Conexï¿½ï¿½es de Mï¿½ï¿½fia (feat. Rich </t>
+    <t xml:space="preserve">Conex?es de M?fia (feat. Rich </t>
   </si>
   <si>
     <t>Shoong! (feat. LISA of BLACKPINK)</t>
@@ -2629,7 +2629,7 @@
     <t>A Veces (feat. Feid)</t>
   </si>
   <si>
-    <t>Cartï¿½ï¿½o B</t>
+    <t>Cart?o B</t>
   </si>
   <si>
     <t>The Heart Part 5</t>
@@ -2689,7 +2689,7 @@
     <t>Phir Aur Kya Chahiye (From "Zara Hatke Zara Bachke")</t>
   </si>
   <si>
-    <t>Donï¿½ï¿½ï¿½t Break My</t>
+    <t>Don't Break My</t>
   </si>
   <si>
     <t>Notice Me</t>
@@ -2785,7 +2785,7 @@
     <t>TULUM</t>
   </si>
   <si>
-    <t xml:space="preserve">I Can See You (Taylorï¿½ï¿½ï¿½s Version) (From The </t>
+    <t xml:space="preserve">I Can See You (Taylor's Version) (From The </t>
   </si>
   <si>
     <t>Lilith (feat. SUGA of BTS) (Diablo IV Anthem)</t>
@@ -2806,7 +2806,7 @@
     <t>Cheques</t>
   </si>
   <si>
-    <t>XQ Te Pones Asï¿</t>
+    <t>XQ Te Pones As?</t>
   </si>
   <si>
     <t>Karma (feat. Ice Spice)</t>
@@ -2815,10 +2815,10 @@
     <t>Stand By Me (feat. Morgan Wallen)</t>
   </si>
   <si>
-    <t>CORAZï¿½ï¿½N VA</t>
-  </si>
-  <si>
-    <t>Piï¿½ï¿½man Deï¿</t>
+    <t>CORAZ?N VA</t>
+  </si>
+  <si>
+    <t>Pi?man De?</t>
   </si>
   <si>
     <t>Crown</t>
@@ -2833,7 +2833,7 @@
     <t>Curtains</t>
   </si>
   <si>
-    <t>Novidade na ï¿½ï¿</t>
+    <t>Novidade na ?</t>
   </si>
   <si>
     <t>Hummingbird (Metro Boomin &amp; James Blake)</t>
@@ -2878,7 +2878,7 @@
     <t>Link Up (Metro Boomin &amp; Don Toliver, Wizkid feat. BEAM &amp; Toian) - Spider-Verse Remix (Spider-Man: Across the Spider-Verse )</t>
   </si>
   <si>
-    <t>Devil Donï¿½ï¿½ï¿½</t>
+    <t>Devil Don'</t>
   </si>
   <si>
     <t>Phantom Regret by Jim</t>
@@ -3115,7 +3115,7 @@
     <t>Alec Benjamin</t>
   </si>
   <si>
-    <t>Mï¿½ï¿½ne</t>
+    <t>Måneskin</t>
   </si>
   <si>
     <t>Coolio, L.V.</t>
@@ -3211,7 +3211,7 @@
     <t>Masked Wolf</t>
   </si>
   <si>
-    <t>Bomba Estï¿½ï¿½reo, Bad B</t>
+    <t>Bomba Estéreo, Bad B</t>
   </si>
   <si>
     <t>One Direction</t>
@@ -3238,7 +3238,7 @@
     <t>Halsey, BTS</t>
   </si>
   <si>
-    <t>Tiï¿½ï¿</t>
+    <t>Tiësto</t>
   </si>
   <si>
     <t>Coldplay, BTS</t>
@@ -3295,7 +3295,7 @@
     <t>Eminem, Dido</t>
   </si>
   <si>
-    <t>Rï¿½ï¿½ma, Selena G</t>
+    <t>Rema, Selena G</t>
   </si>
   <si>
     <t>Jaymes Young</t>
@@ -3307,7 +3307,7 @@
     <t>Karol G</t>
   </si>
   <si>
-    <t>Elley Duhï¿</t>
+    <t>Elley Duhé</t>
   </si>
   <si>
     <t>Riton, Nightcrawlers, Mufasa &amp; Hypeman, Dopamine</t>
@@ -3334,7 +3334,7 @@
     <t>Chencho Corleone, Rauw Alejandro</t>
   </si>
   <si>
-    <t>Michael Bublï¿</t>
+    <t>Michael Bublé</t>
   </si>
   <si>
     <t>Polo G</t>
@@ -3343,7 +3343,7 @@
     <t>Beach House</t>
   </si>
   <si>
-    <t>ROSALï¿½</t>
+    <t>ROSALÍA</t>
   </si>
   <si>
     <t>Julieta Venegas, Bad Bunny, Tainy</t>
@@ -3433,7 +3433,7 @@
     <t>Daddy Yankee</t>
   </si>
   <si>
-    <t>Tiï¿½ï¿½sto, Ava</t>
+    <t>Tiësto, Ava</t>
   </si>
   <si>
     <t>Eminem, Dina Rae</t>
@@ -3484,7 +3484,7 @@
     <t>Tini, Maria Becerra</t>
   </si>
   <si>
-    <t>Beyoncï¿</t>
+    <t>Beyoncé</t>
   </si>
   <si>
     <t>Drake, Project Pat, 21 Savage</t>
@@ -3514,7 +3514,7 @@
     <t>Seafret</t>
   </si>
   <si>
-    <t>Tiï¿½ï¿½sto, Kar</t>
+    <t>Tiësto, Kar</t>
   </si>
   <si>
     <t>Labrinth</t>
@@ -3559,7 +3559,7 @@
     <t>Zion &amp; Lennox</t>
   </si>
   <si>
-    <t>Josï¿½ï¿½ Felic</t>
+    <t>José Feliciano</t>
   </si>
   <si>
     <t>Maluma</t>
@@ -3649,7 +3649,7 @@
     <t>Dean Martin</t>
   </si>
   <si>
-    <t>Rï¿½ï</t>
+    <t>R?</t>
   </si>
   <si>
     <t>Childish Gambino</t>
@@ -3730,7 +3730,7 @@
     <t>Ryan Castro</t>
   </si>
   <si>
-    <t>Justin Quiles, Lenny Tavï¿½ï¿½rez, BL</t>
+    <t>Justin Quiles, Lenny Tavárez, BL</t>
   </si>
   <si>
     <t>Nat King Cole</t>
@@ -3754,7 +3754,7 @@
     <t>PnB Rock</t>
   </si>
   <si>
-    <t>The Weeknd, ROSALï¿½</t>
+    <t>The Weeknd, ROSALÍA</t>
   </si>
   <si>
     <t>Bizarrap, Tiago pzk</t>
@@ -3781,7 +3781,7 @@
     <t>Jimin</t>
   </si>
   <si>
-    <t>Rauw Alejandro, ROSALï¿½</t>
+    <t>Rauw Alejandro, ROSALÍA</t>
   </si>
   <si>
     <t>INTERWORLD</t>
@@ -3835,7 +3835,7 @@
     <t>Intense, AP Dhillon, Gurinder Gill</t>
   </si>
   <si>
-    <t>Tiï¿½ï¿½sto, Tate M</t>
+    <t>Tiësto, Tate M</t>
   </si>
   <si>
     <t>Luis R Conriquez, La Adictiva</t>
@@ -3856,7 +3856,7 @@
     <t>King</t>
   </si>
   <si>
-    <t>Bad Bunny, The Marï¿½ï</t>
+    <t>Bad Bunny, The Marías</t>
   </si>
   <si>
     <t>V</t>
@@ -3865,7 +3865,7 @@
     <t>Young Thug, Future, Gunna</t>
   </si>
   <si>
-    <t>Wisin &amp; Yandel, ROSALï¿½</t>
+    <t>Wisin &amp; Yandel, ROSALÍA</t>
   </si>
   <si>
     <t>Polima WestCoast, Pailita</t>
@@ -3892,7 +3892,7 @@
     <t>MNEK, Jax Jones</t>
   </si>
   <si>
-    <t>Eden Muï¿½ï</t>
+    <t>Eden Muñoz</t>
   </si>
   <si>
     <t>Dua Lipa, Megan Thee Stallion</t>
@@ -3919,7 +3919,7 @@
     <t>Lizzy McAlpine</t>
   </si>
   <si>
-    <t>Marï¿½ï¿½lia Mendonï¿½ï¿½a, Hugo &amp; G</t>
+    <t>Marília Mendonça, Hugo &amp; G</t>
   </si>
   <si>
     <t>NIKI</t>
@@ -3964,7 +3964,7 @@
     <t>Post Malone, Roddy Ricch</t>
   </si>
   <si>
-    <t>Marï¿½ï¿½lia Mendo</t>
+    <t>Marília Mendonça</t>
   </si>
   <si>
     <t>Jessica Darrow</t>
@@ -3973,7 +3973,7 @@
     <t>Karol G, Romeo Santos</t>
   </si>
   <si>
-    <t>Marï¿½ï¿½lia Mendonï¿½ï¿½a, George Henrique &amp;</t>
+    <t>Marília Mendonça, George Henrique &amp;</t>
   </si>
   <si>
     <t>YEAT</t>
@@ -3997,7 +3997,7 @@
     <t>Em Beihold</t>
   </si>
   <si>
-    <t>Marï¿½ï¿½lia Mendonï¿½ï¿½a, Maiara &amp;</t>
+    <t>Marília Mendonça, Maiara &amp;</t>
   </si>
   <si>
     <t>Kali Uchis</t>
@@ -4024,7 +4024,7 @@
     <t>Jung Kook</t>
   </si>
   <si>
-    <t>Quevedo, La Pantera, Juseph, Cruz Cafunï¿½ï¿½, Bï¿½ï¿½jo, Abhir Hathi</t>
+    <t>Quevedo, La Pantera, Juseph, Cruz Cafuné, B?jo, Abhir Hathi</t>
   </si>
   <si>
     <t>Chuck Berry</t>
@@ -4060,7 +4060,7 @@
     <t>Yung Lean</t>
   </si>
   <si>
-    <t>Xamï¿½ï¿½, Gustah, Neo B</t>
+    <t>Xamã, Gustah, Neo B</t>
   </si>
   <si>
     <t>Paulo Londra</t>
@@ -4108,7 +4108,7 @@
     <t>Duki, NICKI NICOLE, Cris Mj, Standly, Stars Music Chile</t>
   </si>
   <si>
-    <t>Arcangel, De La Ghetto, Justin Quiles, Lenny Tavï¿½ï¿½rez, Sech, Dalex, Dimelo Flow, Rich Music</t>
+    <t>Arcangel, De La Ghetto, Justin Quiles, Lenny Tavárez, Sech, Dalex, Dimelo Flow, Rich Music</t>
   </si>
   <si>
     <t>Gustavo Mioto, Mari Fernandez</t>
@@ -4222,7 +4222,7 @@
     <t>Yahritza Y Su Esencia, Grupo Frontera</t>
   </si>
   <si>
-    <t xml:space="preserve">Matuï¿½ï¿½, Wiu, </t>
+    <t xml:space="preserve">Matuê, Wiu, </t>
   </si>
   <si>
     <t>MC Ryan SP, Love Funk, Mc Paiva ZS</t>
@@ -4282,7 +4282,7 @@
     <t>Fuerza Regida</t>
   </si>
   <si>
-    <t>Luï¿½ï¿½sa Sonza, MC Frog, Dj Gabriel do Borel, Davi K</t>
+    <t>Luísa Sonza, MC Frog, Dj Gabriel do Borel, Davi K</t>
   </si>
   <si>
     <t>L7nnon, DJ Biel do Furduncinho, Bianca</t>
@@ -4363,7 +4363,7 @@
     <t>Southstar</t>
   </si>
   <si>
-    <t>Zï¿½ï¿½ Fe</t>
+    <t>Zé Felipe</t>
   </si>
   <si>
     <t>Simone Mendes</t>
@@ -4387,10 +4387,10 @@
     <t>Mambo Kingz, DJ Luian, Anuel Aa</t>
   </si>
   <si>
-    <t>Luciano, Aitch, Bï¿½</t>
-  </si>
-  <si>
-    <t>Zï¿½ï¿½ Neto &amp; Crist</t>
+    <t>Luciano, Aitch, B?</t>
+  </si>
+  <si>
+    <t>Zé Neto &amp; Cristiano</t>
   </si>
   <si>
     <t>Niall Horan</t>
@@ -4471,7 +4471,7 @@
     <t>Nessa Barrett</t>
   </si>
   <si>
-    <t>Schï¿½ï¿½rze, DJ R</t>
+    <t>Schürze, DJ R</t>
   </si>
   <si>
     <t>Mc Vitin Da Igrejinha, MC Tairon, DJ Win</t>
@@ -4510,7 +4510,7 @@
     <t>Steve Aoki, Tini, La Joaqui</t>
   </si>
   <si>
-    <t>Jordan Fisher, Josh Levi, Finneas O'Connell, 4*TOWN (From Disney and Pixarï¿½ï¿½ï¿½s Turning Red), Topher Ngo, Grayson Vill</t>
+    <t>Jordan Fisher, Josh Levi, Finneas O'Connell, 4*TOWN (From Disney and Pixar's Turning Red), Topher Ngo, Grayson Vill</t>
   </si>
   <si>
     <t>Agust D</t>
@@ -4525,7 +4525,7 @@
     <t>Fuerza Regida, Chino Pacas</t>
   </si>
   <si>
-    <t>Dj LK da Escï¿½ï¿½cia, Tchakabum, mc jhenny, M</t>
+    <t>Dj LK da Escócia, Tchakabum, mc jhenny, M</t>
   </si>
   <si>
     <t>The Weeknd, Madonna, Playboi Carti</t>
@@ -4636,16 +4636,16 @@
     <t>SEVENTEEN</t>
   </si>
   <si>
-    <t>Sebastian Yatra, Manuel Turizo, Beï¿½ï</t>
+    <t>Sebastian Yatra, Manuel Turizo, Be?</t>
   </si>
   <si>
     <t>Styrx, utku INC, Thezth</t>
   </si>
   <si>
-    <t>Jasiel Nuï¿½ï¿½ez, Peso P</t>
-  </si>
-  <si>
-    <t>Junior H, Eden Muï¿½ï</t>
+    <t>Jasiel Núñez, Peso P</t>
+  </si>
+  <si>
+    <t>Junior H, Eden Muñoz</t>
   </si>
   <si>
     <t>The Weeknd, Tyler, The Creator</t>
@@ -4684,7 +4684,7 @@
     <t>Carin Leon</t>
   </si>
   <si>
-    <t>Rich The Kid, Matuï¿</t>
+    <t>Rich The Kid, Matuê</t>
   </si>
   <si>
     <t>TAEYANG, Lisa</t>
@@ -4765,7 +4765,7 @@
     <t>Feid, Mora, Saiko, Quevedo</t>
   </si>
   <si>
-    <t>Kendrick Lamar, Beyoncï¿</t>
+    <t>Kendrick Lamar, Beyoncé</t>
   </si>
   <si>
     <t>Gunna, Lil Baby</t>
@@ -4804,7 +4804,7 @@
     <t>Maria Becerra</t>
   </si>
   <si>
-    <t xml:space="preserve">Semicenk, Doï¿½ï¿½u </t>
+    <t xml:space="preserve">Semicenk, Doğu </t>
   </si>
   <si>
     <t>Mc Livinho, DJ Matt D</t>

</xml_diff>